<commit_message>
Improve markers and annotations for multi-agent setups
</commit_message>
<xml_diff>
--- a/src/flychams_common/config/Configuration-Multi-Agent.xlsx
+++ b/src/flychams_common/config/Configuration-Multi-Agent.xlsx
@@ -817,7 +817,7 @@
     <numFmt numFmtId="165" formatCode="h:mm:ss"/>
     <numFmt numFmtId="166" formatCode="0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -885,13 +885,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="16"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -985,7 +978,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1036,10 +1029,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1701,7 +1690,7 @@
       <c r="BD3" s="12"/>
     </row>
     <row r="4" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="8" t="s">
         <v>21</v>
       </c>
       <c r="B4" s="9" t="s">
@@ -1899,92 +1888,92 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>249</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>250</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>251</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>252</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>253</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="20" t="s">
         <v>254</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="20" t="s">
         <v>234</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="20" t="s">
         <v>235</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="20" t="s">
         <v>236</v>
       </c>
       <c r="L2" s="12"/>
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>255</v>
       </c>
-      <c r="C3" s="22" t="b">
+      <c r="C3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="21" t="s">
         <v>256</v>
       </c>
-      <c r="E3" s="22" t="b">
+      <c r="E3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="21" t="s">
         <v>257</v>
       </c>
-      <c r="G3" s="22" t="b">
+      <c r="G3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="I3" s="22" t="n">
+      <c r="I3" s="21" t="n">
         <v>0.4</v>
       </c>
-      <c r="J3" s="22" t="n">
+      <c r="J3" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="K3" s="22" t="n">
+      <c r="K3" s="21" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2038,12 +2027,12 @@
   </cols>
   <sheetData>
     <row r="1" s="7" customFormat="true" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
       <c r="E1" s="12"/>
       <c r="XFB1" s="3"/>
       <c r="XFC1" s="3"/>
@@ -2073,7 +2062,7 @@
       <c r="C3" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="14" t="s">
         <v>32</v>
       </c>
     </row>
@@ -2087,7 +2076,7 @@
       <c r="C4" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="14" t="s">
         <v>35</v>
       </c>
     </row>
@@ -2127,15 +2116,15 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
@@ -2231,7 +2220,7 @@
       <c r="D3" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="16" t="n">
+      <c r="E3" s="15" t="n">
         <v>2</v>
       </c>
       <c r="F3" s="9" t="s">
@@ -2312,7 +2301,7 @@
       <c r="D4" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="16" t="n">
+      <c r="E4" s="15" t="n">
         <v>4</v>
       </c>
       <c r="F4" s="9" t="s">
@@ -2393,7 +2382,7 @@
       <c r="D5" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="15" t="n">
         <v>8</v>
       </c>
       <c r="F5" s="9" t="s">
@@ -2474,7 +2463,7 @@
       <c r="D6" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="15" t="n">
         <v>16</v>
       </c>
       <c r="F6" s="9" t="s">
@@ -2587,48 +2576,48 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="17" t="s">
         <v>64</v>
       </c>
       <c r="L2" s="12"/>
@@ -2643,258 +2632,258 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="H3" s="19" t="n">
+      <c r="H3" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I3" s="19" t="n">
+      <c r="I3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="19" t="n">
+      <c r="J3" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="H4" s="19" t="n">
+      <c r="H4" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I4" s="19" t="n">
+      <c r="I4" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="19" t="n">
+      <c r="J4" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="H5" s="19" t="n">
+      <c r="H5" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I5" s="19" t="n">
+      <c r="I5" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J5" s="19" t="n">
+      <c r="J5" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="H6" s="19" t="n">
+      <c r="H6" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I6" s="19" t="n">
+      <c r="I6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="19" t="n">
+      <c r="J6" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="H7" s="19" t="n">
+      <c r="H7" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I7" s="19" t="n">
+      <c r="I7" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J7" s="19" t="n">
+      <c r="J7" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="H8" s="19" t="n">
+      <c r="H8" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="I8" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="19" t="n">
+      <c r="J8" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="H9" s="19" t="n">
+      <c r="H9" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="I9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="J9" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="G10" s="19" t="s">
+      <c r="G10" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="H10" s="19" t="n">
+      <c r="H10" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="I10" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J10" s="19" t="n">
+      <c r="J10" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -2940,32 +2929,32 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>97</v>
       </c>
       <c r="H2" s="12"/>
@@ -2981,22 +2970,22 @@
       <c r="XFD2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="D3" s="19" t="n">
+      <c r="D3" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E3" s="19" t="n">
+      <c r="E3" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F3" s="19" t="n">
+      <c r="F3" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G3" s="2"/>
@@ -3006,22 +2995,22 @@
       <c r="XEY3" s="3"/>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D4" s="19" t="n">
+      <c r="D4" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="19" t="n">
+      <c r="E4" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F4" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G4" s="2"/>
@@ -3036,22 +3025,22 @@
       <c r="XFD4" s="3"/>
     </row>
     <row r="5" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F5" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G5" s="2"/>
@@ -3066,22 +3055,22 @@
       <c r="XFD5" s="3"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F6" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G6" s="2"/>
@@ -3091,22 +3080,22 @@
       <c r="XEY6" s="3"/>
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F7" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G7" s="2"/>
@@ -3116,22 +3105,22 @@
       <c r="XEY7" s="3"/>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E8" s="19" t="n">
+      <c r="E8" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F8" s="19" t="n">
+      <c r="F8" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G8" s="2"/>
@@ -3141,22 +3130,22 @@
       <c r="XEY8" s="3"/>
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G9" s="2"/>
@@ -3166,22 +3155,22 @@
       <c r="XEY9" s="3"/>
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E10" s="19" t="n">
+      <c r="E10" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F10" s="19" t="n">
+      <c r="F10" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G10" s="2"/>
@@ -3247,56 +3236,56 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="K2" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="L2" s="18" t="s">
+      <c r="L2" s="17" t="s">
         <v>120</v>
       </c>
       <c r="M2" s="12"/>
@@ -3309,648 +3298,648 @@
       <c r="XFC2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="I3" s="19" t="n">
+      <c r="I3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="19" t="n">
+      <c r="J3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K3" s="19" t="n">
+      <c r="K3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L3" s="19" t="s">
+      <c r="L3" s="18" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>130</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="H4" s="19" t="s">
+      <c r="H4" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="I4" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="J4" s="19" t="n">
+      <c r="I4" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K4" s="19" t="n">
+      <c r="K4" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L4" s="19" t="s">
+      <c r="L4" s="18" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>137</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="I5" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="J5" s="19" t="n">
+      <c r="I5" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K5" s="19" t="n">
+      <c r="K5" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L5" s="19" t="s">
+      <c r="L5" s="18" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H6" s="19" t="s">
+      <c r="H6" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="I6" s="19" t="n">
+      <c r="I6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="19" t="n">
+      <c r="J6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K6" s="19" t="n">
+      <c r="K6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L6" s="19" t="s">
+      <c r="L6" s="18" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>144</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="H7" s="19" t="s">
+      <c r="H7" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="I7" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="J7" s="19" t="n">
+      <c r="I7" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K7" s="19" t="n">
+      <c r="K7" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L7" s="19" t="s">
+      <c r="L7" s="18" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="H8" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="I8" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="J8" s="19" t="n">
+      <c r="I8" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K8" s="19" t="n">
+      <c r="K8" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L8" s="19" t="s">
+      <c r="L8" s="18" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H9" s="19" t="s">
+      <c r="H9" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="I9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="J9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K9" s="19" t="n">
+      <c r="K9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L9" s="19" t="s">
+      <c r="L9" s="18" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="G10" s="19" t="s">
+      <c r="G10" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="H10" s="19" t="s">
+      <c r="H10" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="I10" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="J10" s="19" t="n">
+      <c r="I10" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K10" s="19" t="n">
+      <c r="K10" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L10" s="19" t="s">
+      <c r="L10" s="18" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="11" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H11" s="19" t="s">
+      <c r="H11" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="I11" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="J11" s="19" t="n">
+      <c r="I11" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K11" s="19" t="n">
+      <c r="K11" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L11" s="19" t="s">
+      <c r="L11" s="18" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E12" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F12" s="19" t="s">
+      <c r="F12" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="G12" s="19" t="s">
+      <c r="G12" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H12" s="19" t="s">
+      <c r="H12" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="I12" s="19" t="n">
+      <c r="I12" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J12" s="19" t="n">
+      <c r="J12" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K12" s="19" t="n">
+      <c r="K12" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L12" s="19" t="s">
+      <c r="L12" s="18" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F13" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H13" s="19" t="s">
+      <c r="H13" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="I13" s="19" t="n">
+      <c r="I13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J13" s="19" t="n">
+      <c r="J13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K13" s="19" t="n">
+      <c r="K13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L13" s="19" t="s">
+      <c r="L13" s="18" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="18" t="s">
         <v>165</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F14" s="19" t="s">
+      <c r="F14" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="G14" s="19" t="s">
+      <c r="G14" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H14" s="19" t="s">
+      <c r="H14" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="I14" s="19" t="n">
+      <c r="I14" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J14" s="19" t="n">
+      <c r="J14" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K14" s="19" t="n">
+      <c r="K14" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L14" s="19" t="s">
+      <c r="L14" s="18" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="E15" s="19" t="s">
+      <c r="E15" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F15" s="19" t="s">
+      <c r="F15" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="G15" s="19" t="s">
+      <c r="G15" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H15" s="19" t="s">
+      <c r="H15" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="I15" s="19" t="n">
+      <c r="I15" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J15" s="19" t="n">
+      <c r="J15" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K15" s="19" t="n">
+      <c r="K15" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L15" s="19" t="s">
+      <c r="L15" s="18" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="18" t="s">
         <v>171</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="18" t="s">
         <v>172</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="C16" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D16" s="19" t="s">
+      <c r="D16" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E16" s="19" t="s">
+      <c r="E16" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F16" s="19" t="s">
+      <c r="F16" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="G16" s="19" t="s">
+      <c r="G16" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="H16" s="19" t="s">
+      <c r="H16" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="I16" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="J16" s="19" t="n">
+      <c r="I16" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K16" s="19" t="n">
+      <c r="K16" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L16" s="19" t="s">
+      <c r="L16" s="18" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="18" t="s">
         <v>174</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="C17" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D17" s="19" t="s">
+      <c r="D17" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E17" s="19" t="s">
+      <c r="E17" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F17" s="19" t="s">
+      <c r="F17" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="G17" s="19" t="s">
+      <c r="G17" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="H17" s="19" t="s">
+      <c r="H17" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="I17" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="J17" s="19" t="n">
+      <c r="I17" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K17" s="19" t="n">
+      <c r="K17" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L17" s="19" t="s">
+      <c r="L17" s="18" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D18" s="19" t="s">
+      <c r="D18" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E18" s="19" t="s">
+      <c r="E18" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F18" s="19" t="s">
+      <c r="F18" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="G18" s="19" t="s">
+      <c r="G18" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="H18" s="19" t="s">
+      <c r="H18" s="18" t="s">
         <v>180</v>
       </c>
-      <c r="I18" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="J18" s="19" t="n">
+      <c r="I18" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K18" s="19" t="n">
+      <c r="K18" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L18" s="19" t="s">
+      <c r="L18" s="18" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="18" t="s">
         <v>182</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="C19" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D19" s="19" t="s">
+      <c r="D19" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="E19" s="19" t="s">
+      <c r="E19" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F19" s="19" t="s">
+      <c r="F19" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="G19" s="19" t="s">
+      <c r="G19" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H19" s="19" t="s">
+      <c r="H19" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="I19" s="19" t="n">
+      <c r="I19" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J19" s="19" t="n">
+      <c r="J19" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K19" s="19" t="n">
+      <c r="K19" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L19" s="19" t="s">
+      <c r="L19" s="18" t="s">
         <v>184</v>
       </c>
     </row>
@@ -3991,36 +3980,36 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>186</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>188</v>
       </c>
       <c r="XEU2" s="3"/>
@@ -4035,209 +4024,209 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>189</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>190</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="E3" s="19" t="n">
+      <c r="E3" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F3" s="19" t="n">
+      <c r="F3" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="19" t="n">
+      <c r="G3" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>192</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="E4" s="19" t="n">
+      <c r="E4" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F4" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="19" t="n">
+      <c r="G4" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F5" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="19" t="n">
+      <c r="G5" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>196</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F6" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="19" t="n">
+      <c r="G6" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>198</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>199</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F7" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="19" t="n">
+      <c r="G7" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>200</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>201</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="E8" s="19" t="n">
+      <c r="E8" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F8" s="19" t="n">
+      <c r="F8" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="19" t="n">
+      <c r="G8" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>202</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>203</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="19" t="n">
+      <c r="G9" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="E10" s="19" t="n">
+      <c r="E10" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F10" s="19" t="n">
+      <c r="F10" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="19" t="n">
+      <c r="G10" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="18" t="s">
         <v>206</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="18" t="s">
         <v>207</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="E11" s="19" t="n">
+      <c r="E11" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F11" s="19" t="n">
+      <c r="F11" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="19" t="n">
+      <c r="G11" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
@@ -4288,140 +4277,140 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="20"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
+      <c r="P1" s="19"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="19"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>209</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>210</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>211</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>212</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="20" t="s">
         <v>213</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="20" t="s">
         <v>214</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="20" t="s">
         <v>215</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="20" t="s">
         <v>216</v>
       </c>
-      <c r="L2" s="21" t="s">
+      <c r="L2" s="20" t="s">
         <v>217</v>
       </c>
-      <c r="M2" s="21" t="s">
+      <c r="M2" s="20" t="s">
         <v>218</v>
       </c>
-      <c r="N2" s="21" t="s">
+      <c r="N2" s="20" t="s">
         <v>219</v>
       </c>
-      <c r="O2" s="21" t="s">
+      <c r="O2" s="20" t="s">
         <v>220</v>
       </c>
-      <c r="P2" s="21" t="s">
+      <c r="P2" s="20" t="s">
         <v>221</v>
       </c>
-      <c r="Q2" s="21" t="s">
+      <c r="Q2" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="R2" s="21" t="s">
+      <c r="R2" s="20" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>224</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="21" t="s">
         <v>225</v>
       </c>
-      <c r="D3" s="22" t="n">
+      <c r="D3" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="E3" s="22" t="n">
+      <c r="E3" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="F3" s="22" t="b">
+      <c r="F3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="G3" s="21" t="s">
         <v>226</v>
       </c>
-      <c r="H3" s="22" t="b">
+      <c r="H3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="I3" s="22" t="s">
+      <c r="I3" s="21" t="s">
         <v>227</v>
       </c>
-      <c r="J3" s="22" t="b">
+      <c r="J3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="K3" s="22" t="s">
+      <c r="K3" s="21" t="s">
         <v>228</v>
       </c>
-      <c r="L3" s="22" t="b">
+      <c r="L3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="M3" s="22" t="s">
+      <c r="M3" s="21" t="s">
         <v>229</v>
       </c>
-      <c r="N3" s="22" t="n">
+      <c r="N3" s="21" t="n">
         <v>6.5</v>
       </c>
-      <c r="O3" s="22" t="n">
+      <c r="O3" s="21" t="n">
         <v>2.5</v>
       </c>
-      <c r="P3" s="22" t="n">
+      <c r="P3" s="21" t="n">
         <v>400</v>
       </c>
-      <c r="Q3" s="22" t="n">
+      <c r="Q3" s="21" t="n">
         <v>350</v>
       </c>
-      <c r="R3" s="22" t="n">
+      <c r="R3" s="21" t="n">
         <v>25</v>
       </c>
     </row>
@@ -4481,52 +4470,52 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>185</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>230</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>231</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>232</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="20" t="s">
         <v>233</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="20" t="s">
         <v>234</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="20" t="s">
         <v>235</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="20" t="s">
         <v>236</v>
       </c>
       <c r="XFB2" s="3"/>
@@ -4534,110 +4523,110 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>237</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="E3" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="G3" s="22" t="b">
+      <c r="G3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="I3" s="22" t="n">
+      <c r="I3" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="J3" s="22" t="n">
+      <c r="J3" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K3" s="22" t="n">
+      <c r="K3" s="21" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="21" t="s">
         <v>243</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="21" t="s">
         <v>244</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="F4" s="22" t="s">
+      <c r="F4" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="G4" s="22" t="b">
+      <c r="G4" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H4" s="22" t="s">
+      <c r="H4" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="I4" s="22" t="n">
+      <c r="I4" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="J4" s="22" t="n">
+      <c r="J4" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="22" t="n">
+      <c r="K4" s="21" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>160</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="21" t="s">
         <v>245</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="21" t="s">
         <v>246</v>
       </c>
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="F5" s="22" t="s">
+      <c r="F5" s="21" t="s">
         <v>247</v>
       </c>
-      <c r="G5" s="22" t="b">
+      <c r="G5" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H5" s="22" t="s">
+      <c r="H5" s="21" t="s">
         <v>248</v>
       </c>
-      <c r="I5" s="22" t="n">
+      <c r="I5" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="J5" s="22" t="n">
+      <c r="J5" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="22" t="n">
+      <c r="K5" s="21" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Launch agent assignment asynchronously
</commit_message>
<xml_diff>
--- a/src/flychams_common/config/Configuration-Multi-Agent.xlsx
+++ b/src/flychams_common/config/Configuration-Multi-Agent.xlsx
@@ -73,120 +73,123 @@
     <t xml:space="preserve">ENVIRONMENT00</t>
   </si>
   <si>
+    <t xml:space="preserve">GROUP03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEAM00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(-150.0, 150.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(30.0, 150.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PX4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(13/12/2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(16:30:00)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MISSION01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Homogeneus Configuration (B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEAM01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MISSION02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heterogeneus Configuration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEAM02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geopoint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WindVel [m/s]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operational Conditions O1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(lat=35.9865559, lon=-5.8930106, alt=0.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(Vx=3.0, Vy=1.5, Vz=0.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENVIRONMENT01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operational Conditions O2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(Vx=4.0, Vy=3.5, Vz=0.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Priority</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TrajectoryFolder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TARGET00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target Configuration L1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GROUP00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Human</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TargetConfigurationL1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TARGET01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target Configuration L2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GROUP01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TargetConfigurationL2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TARGET02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target Configuration L3</t>
+  </si>
+  <si>
     <t xml:space="preserve">GROUP02</t>
   </si>
   <si>
-    <t xml:space="preserve">TEAM00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(-150.0, 150.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(30.0, 150.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PX4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(13/12/2024)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(16:30:00)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MISSION01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Homogeneus Configuration (B)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEAM01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MISSION02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Heterogeneus Configuration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEAM02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Geopoint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WindVel [m/s]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operational Conditions O1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(lat=35.9865559, lon=-5.8930106, alt=0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(Vx=3.0, Vy=1.5, Vz=0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ENVIRONMENT01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operational Conditions O2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(Vx=4.0, Vy=3.5, Vz=0.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Priority</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TrajectoryFolder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TARGET00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target Configuration L1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GROUP00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Human</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TargetConfigurationL1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TARGET01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target Configuration L2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GROUP01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TargetConfigurationL2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TARGET02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target Configuration L3</t>
-  </si>
-  <si>
     <t xml:space="preserve">TargetConfigurationL3</t>
   </si>
   <si>
@@ -194,9 +197,6 @@
   </si>
   <si>
     <t xml:space="preserve">Target Configuration L4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GROUP03</t>
   </si>
   <si>
     <t xml:space="preserve">TargetConfigurationL4</t>
@@ -2377,7 +2377,7 @@
         <v>51</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>43</v>
@@ -2389,7 +2389,7 @@
         <v>44</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H5" s="12"/>
       <c r="I5" s="12"/>
@@ -2452,13 +2452,13 @@
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>43</v>

</xml_diff>

<commit_message>
Create trajectory generation MATLAB script
</commit_message>
<xml_diff>
--- a/src/flychams_common/config/Configuration-Multi-Agent.xlsx
+++ b/src/flychams_common/config/Configuration-Multi-Agent.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="247">
   <si>
     <t xml:space="preserve">GENERAL CONFIGURATION</t>
   </si>
@@ -73,7 +73,7 @@
     <t xml:space="preserve">ENVIRONMENT00</t>
   </si>
   <si>
-    <t xml:space="preserve">GROUP03</t>
+    <t xml:space="preserve">GROUP00</t>
   </si>
   <si>
     <t xml:space="preserve">TEAM00</t>
@@ -154,10 +154,7 @@
     <t xml:space="preserve">TARGET00</t>
   </si>
   <si>
-    <t xml:space="preserve">Target Configuration L1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GROUP00</t>
+    <t xml:space="preserve">Complex Configuration (6 Clusters)</t>
   </si>
   <si>
     <t xml:space="preserve">Human</t>
@@ -166,40 +163,7 @@
     <t xml:space="preserve">High</t>
   </si>
   <si>
-    <t xml:space="preserve">TargetConfigurationL1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TARGET01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target Configuration L2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GROUP01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TargetConfigurationL2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TARGET02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target Configuration L3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GROUP02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TargetConfigurationL3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TARGET03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target Configuration L4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TargetConfigurationL4</t>
+    <t xml:space="preserve">Complex</t>
   </si>
   <si>
     <t xml:space="preserve">AGENT CONFIGURATION</t>
@@ -1889,7 +1853,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1910,62 +1874,62 @@
         <v>2</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>249</v>
+        <v>237</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="I2" s="20" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="J2" s="20" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="K2" s="20" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="L2" s="12"/>
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="C3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="E3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="G3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H3" s="21" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="I3" s="21" t="n">
         <v>0.4</v>
@@ -2215,19 +2179,19 @@
         <v>41</v>
       </c>
       <c r="C3" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="F3" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" s="9" t="s">
+      <c r="G3" s="9" t="s">
         <v>44</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>45</v>
       </c>
       <c r="H3" s="12"/>
       <c r="I3" s="12"/>
@@ -2288,249 +2252,9 @@
       <c r="BL3" s="12"/>
       <c r="BM3" s="3"/>
     </row>
-    <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E4" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="12"/>
-      <c r="K4" s="12"/>
-      <c r="L4" s="12"/>
-      <c r="M4" s="12"/>
-      <c r="N4" s="12"/>
-      <c r="O4" s="12"/>
-      <c r="P4" s="12"/>
-      <c r="Q4" s="12"/>
-      <c r="R4" s="12"/>
-      <c r="S4" s="12"/>
-      <c r="T4" s="12"/>
-      <c r="U4" s="12"/>
-      <c r="V4" s="12"/>
-      <c r="W4" s="12"/>
-      <c r="X4" s="12"/>
-      <c r="Y4" s="12"/>
-      <c r="Z4" s="12"/>
-      <c r="AA4" s="12"/>
-      <c r="AB4" s="12"/>
-      <c r="AC4" s="12"/>
-      <c r="AD4" s="12"/>
-      <c r="AE4" s="12"/>
-      <c r="AF4" s="12"/>
-      <c r="AG4" s="12"/>
-      <c r="AH4" s="12"/>
-      <c r="AI4" s="12"/>
-      <c r="AJ4" s="12"/>
-      <c r="AK4" s="12"/>
-      <c r="AL4" s="12"/>
-      <c r="AM4" s="12"/>
-      <c r="AN4" s="12"/>
-      <c r="AO4" s="12"/>
-      <c r="AP4" s="12"/>
-      <c r="AQ4" s="12"/>
-      <c r="AR4" s="12"/>
-      <c r="AS4" s="12"/>
-      <c r="AT4" s="12"/>
-      <c r="AU4" s="12"/>
-      <c r="AV4" s="12"/>
-      <c r="AW4" s="12"/>
-      <c r="AX4" s="12"/>
-      <c r="AY4" s="12"/>
-      <c r="AZ4" s="12"/>
-      <c r="BA4" s="12"/>
-      <c r="BB4" s="12"/>
-      <c r="BC4" s="12"/>
-      <c r="BD4" s="12"/>
-      <c r="BE4" s="12"/>
-      <c r="BF4" s="12"/>
-      <c r="BG4" s="12"/>
-      <c r="BH4" s="12"/>
-      <c r="BI4" s="12"/>
-      <c r="BJ4" s="12"/>
-      <c r="BK4" s="12"/>
-      <c r="BL4" s="12"/>
-      <c r="BM4" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E5" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
-      <c r="N5" s="12"/>
-      <c r="O5" s="12"/>
-      <c r="P5" s="12"/>
-      <c r="Q5" s="12"/>
-      <c r="R5" s="12"/>
-      <c r="S5" s="12"/>
-      <c r="T5" s="12"/>
-      <c r="U5" s="12"/>
-      <c r="V5" s="12"/>
-      <c r="W5" s="12"/>
-      <c r="X5" s="12"/>
-      <c r="Y5" s="12"/>
-      <c r="Z5" s="12"/>
-      <c r="AA5" s="12"/>
-      <c r="AB5" s="12"/>
-      <c r="AC5" s="12"/>
-      <c r="AD5" s="12"/>
-      <c r="AE5" s="12"/>
-      <c r="AF5" s="12"/>
-      <c r="AG5" s="12"/>
-      <c r="AH5" s="12"/>
-      <c r="AI5" s="12"/>
-      <c r="AJ5" s="12"/>
-      <c r="AK5" s="12"/>
-      <c r="AL5" s="12"/>
-      <c r="AM5" s="12"/>
-      <c r="AN5" s="12"/>
-      <c r="AO5" s="12"/>
-      <c r="AP5" s="12"/>
-      <c r="AQ5" s="12"/>
-      <c r="AR5" s="12"/>
-      <c r="AS5" s="12"/>
-      <c r="AT5" s="12"/>
-      <c r="AU5" s="12"/>
-      <c r="AV5" s="12"/>
-      <c r="AW5" s="12"/>
-      <c r="AX5" s="12"/>
-      <c r="AY5" s="12"/>
-      <c r="AZ5" s="12"/>
-      <c r="BA5" s="12"/>
-      <c r="BB5" s="12"/>
-      <c r="BC5" s="12"/>
-      <c r="BD5" s="12"/>
-      <c r="BE5" s="12"/>
-      <c r="BF5" s="12"/>
-      <c r="BG5" s="12"/>
-      <c r="BH5" s="12"/>
-      <c r="BI5" s="12"/>
-      <c r="BJ5" s="12"/>
-      <c r="BK5" s="12"/>
-      <c r="BL5" s="12"/>
-      <c r="BM5" s="3"/>
-    </row>
-    <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E6" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="12"/>
-      <c r="N6" s="12"/>
-      <c r="O6" s="12"/>
-      <c r="P6" s="12"/>
-      <c r="Q6" s="12"/>
-      <c r="R6" s="12"/>
-      <c r="S6" s="12"/>
-      <c r="T6" s="12"/>
-      <c r="U6" s="12"/>
-      <c r="V6" s="12"/>
-      <c r="W6" s="12"/>
-      <c r="X6" s="12"/>
-      <c r="Y6" s="12"/>
-      <c r="Z6" s="12"/>
-      <c r="AA6" s="12"/>
-      <c r="AB6" s="12"/>
-      <c r="AC6" s="12"/>
-      <c r="AD6" s="12"/>
-      <c r="AE6" s="12"/>
-      <c r="AF6" s="12"/>
-      <c r="AG6" s="12"/>
-      <c r="AH6" s="12"/>
-      <c r="AI6" s="12"/>
-      <c r="AJ6" s="12"/>
-      <c r="AK6" s="12"/>
-      <c r="AL6" s="12"/>
-      <c r="AM6" s="12"/>
-      <c r="AN6" s="12"/>
-      <c r="AO6" s="12"/>
-      <c r="AP6" s="12"/>
-      <c r="AQ6" s="12"/>
-      <c r="AR6" s="12"/>
-      <c r="AS6" s="12"/>
-      <c r="AT6" s="12"/>
-      <c r="AU6" s="12"/>
-      <c r="AV6" s="12"/>
-      <c r="AW6" s="12"/>
-      <c r="AX6" s="12"/>
-      <c r="AY6" s="12"/>
-      <c r="AZ6" s="12"/>
-      <c r="BA6" s="12"/>
-      <c r="BB6" s="12"/>
-      <c r="BC6" s="12"/>
-      <c r="BD6" s="12"/>
-      <c r="BE6" s="12"/>
-      <c r="BF6" s="12"/>
-      <c r="BG6" s="12"/>
-      <c r="BH6" s="12"/>
-      <c r="BI6" s="12"/>
-      <c r="BJ6" s="12"/>
-      <c r="BK6" s="12"/>
-      <c r="BL6" s="12"/>
-      <c r="BM6" s="3"/>
-    </row>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2577,7 +2301,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -2600,25 +2324,25 @@
         <v>5</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="I2" s="17" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="J2" s="17" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="L2" s="12"/>
       <c r="M2" s="12"/>
@@ -2633,25 +2357,25 @@
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="C3" s="18" t="s">
         <v>15</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="G3" s="18" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="H3" s="18" t="n">
         <v>300</v>
@@ -2665,25 +2389,25 @@
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="C4" s="18" t="s">
         <v>15</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="H4" s="18" t="n">
         <v>300</v>
@@ -2697,25 +2421,25 @@
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="C5" s="18" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="H5" s="18" t="n">
         <v>300</v>
@@ -2729,25 +2453,25 @@
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="C6" s="18" t="s">
         <v>24</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="H6" s="18" t="n">
         <v>300</v>
@@ -2761,25 +2485,25 @@
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="C7" s="18" t="s">
         <v>24</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="H7" s="18" t="n">
         <v>300</v>
@@ -2793,25 +2517,25 @@
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="C8" s="18" t="s">
         <v>24</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="H8" s="18" t="n">
         <v>300</v>
@@ -2825,25 +2549,25 @@
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="C9" s="18" t="s">
         <v>27</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="H9" s="18" t="n">
         <v>300</v>
@@ -2857,25 +2581,25 @@
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="C10" s="18" t="s">
         <v>27</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="H10" s="18" t="n">
         <v>300</v>
@@ -2930,7 +2654,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -2946,16 +2670,16 @@
         <v>2</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="H2" s="12"/>
       <c r="I2" s="12"/>
@@ -2971,13 +2695,13 @@
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="D3" s="18" t="n">
         <v>0.2</v>
@@ -2996,13 +2720,13 @@
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D4" s="18" t="n">
         <v>0.2</v>
@@ -3018,21 +2742,16 @@
       <c r="XEW4" s="2"/>
       <c r="XEX4" s="2"/>
       <c r="XEY4" s="3"/>
-      <c r="XEZ4" s="3"/>
-      <c r="XFA4" s="3"/>
-      <c r="XFB4" s="3"/>
-      <c r="XFC4" s="3"/>
-      <c r="XFD4" s="3"/>
     </row>
     <row r="5" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="D5" s="18" t="n">
         <v>0.2</v>
@@ -3048,21 +2767,16 @@
       <c r="XEW5" s="2"/>
       <c r="XEX5" s="2"/>
       <c r="XEY5" s="3"/>
-      <c r="XEZ5" s="3"/>
-      <c r="XFA5" s="3"/>
-      <c r="XFB5" s="3"/>
-      <c r="XFC5" s="3"/>
-      <c r="XFD5" s="3"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="D6" s="18" t="n">
         <v>0.2</v>
@@ -3081,13 +2795,13 @@
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="D7" s="18" t="n">
         <v>0.2</v>
@@ -3106,13 +2820,13 @@
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="D8" s="18" t="n">
         <v>0.2</v>
@@ -3131,13 +2845,13 @@
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="D9" s="18" t="n">
         <v>0.2</v>
@@ -3156,13 +2870,13 @@
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="D10" s="18" t="n">
         <v>0.2</v>
@@ -3217,7 +2931,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:XFC19"/>
+  <dimension ref="A1:XFD19"/>
   <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.35"/>
@@ -3237,7 +2951,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -3259,34 +2973,34 @@
         <v>2</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="I2" s="17" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="J2" s="17" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="K2" s="17" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="L2" s="17" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="M2" s="12"/>
       <c r="N2" s="12"/>
@@ -3299,28 +3013,28 @@
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="G3" s="18" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="H3" s="18" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I3" s="18" t="n">
         <v>3</v>
@@ -3332,33 +3046,33 @@
         <v>3</v>
       </c>
       <c r="L3" s="18" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="I4" s="18" t="n">
         <v>1</v>
@@ -3370,33 +3084,33 @@
         <v>10</v>
       </c>
       <c r="L4" s="18" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I5" s="18" t="n">
         <v>1</v>
@@ -3408,33 +3122,34 @@
         <v>10</v>
       </c>
       <c r="L5" s="18" t="s">
-        <v>139</v>
-      </c>
+        <v>127</v>
+      </c>
+      <c r="XFD5" s="12"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="H6" s="18" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I6" s="18" t="n">
         <v>3</v>
@@ -3446,33 +3161,33 @@
         <v>3</v>
       </c>
       <c r="L6" s="18" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="I7" s="18" t="n">
         <v>1</v>
@@ -3484,33 +3199,33 @@
         <v>10</v>
       </c>
       <c r="L7" s="18" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="H8" s="18" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I8" s="18" t="n">
         <v>1</v>
@@ -3522,33 +3237,33 @@
         <v>10</v>
       </c>
       <c r="L8" s="18" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="H9" s="18" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I9" s="18" t="n">
         <v>3</v>
@@ -3560,33 +3275,34 @@
         <v>3</v>
       </c>
       <c r="L9" s="18" t="s">
-        <v>151</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="XFD9" s="2"/>
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="H10" s="18" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="I10" s="18" t="n">
         <v>1</v>
@@ -3598,33 +3314,34 @@
         <v>10</v>
       </c>
       <c r="L10" s="18" t="s">
-        <v>154</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="XFD10" s="2"/>
     </row>
     <row r="11" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="G11" s="18" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="H11" s="18" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I11" s="18" t="n">
         <v>1</v>
@@ -3636,33 +3353,34 @@
         <v>10</v>
       </c>
       <c r="L11" s="18" t="s">
-        <v>157</v>
-      </c>
+        <v>145</v>
+      </c>
+      <c r="XFD11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="H12" s="18" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I12" s="18" t="n">
         <v>3</v>
@@ -3674,33 +3392,33 @@
         <v>3</v>
       </c>
       <c r="L12" s="18" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="H13" s="18" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I13" s="18" t="n">
         <v>3</v>
@@ -3712,33 +3430,33 @@
         <v>3</v>
       </c>
       <c r="L13" s="18" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="H14" s="18" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I14" s="18" t="n">
         <v>3</v>
@@ -3750,33 +3468,33 @@
         <v>3</v>
       </c>
       <c r="L14" s="18" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="C15" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="D15" s="18" t="s">
-        <v>123</v>
-      </c>
       <c r="E15" s="18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="H15" s="18" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I15" s="18" t="n">
         <v>3</v>
@@ -3788,33 +3506,33 @@
         <v>3</v>
       </c>
       <c r="L15" s="18" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="H16" s="18" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="I16" s="18" t="n">
         <v>1</v>
@@ -3826,33 +3544,33 @@
         <v>10</v>
       </c>
       <c r="L16" s="18" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="G17" s="18" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="H17" s="18" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I17" s="18" t="n">
         <v>1</v>
@@ -3864,33 +3582,33 @@
         <v>10</v>
       </c>
       <c r="L17" s="18" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="H18" s="18" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="I18" s="18" t="n">
         <v>1</v>
@@ -3902,33 +3620,33 @@
         <v>10</v>
       </c>
       <c r="L18" s="18" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="C19" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="F19" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D19" s="18" t="s">
-        <v>160</v>
-      </c>
-      <c r="E19" s="18" t="s">
-        <v>124</v>
-      </c>
-      <c r="F19" s="18" t="s">
-        <v>125</v>
-      </c>
       <c r="G19" s="18" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="H19" s="18" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I19" s="18" t="n">
         <v>3</v>
@@ -3940,7 +3658,7 @@
         <v>3</v>
       </c>
       <c r="L19" s="18" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -3981,7 +3699,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -3998,19 +3716,19 @@
         <v>2</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="XEU2" s="3"/>
       <c r="XEV2" s="3"/>
@@ -4025,16 +3743,16 @@
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="E3" s="18" t="n">
         <v>0.167</v>
@@ -4048,16 +3766,16 @@
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="E4" s="18" t="n">
         <v>0.167</v>
@@ -4071,16 +3789,16 @@
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="E5" s="18" t="n">
         <v>0.167</v>
@@ -4094,16 +3812,16 @@
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="E6" s="18" t="n">
         <v>0.167</v>
@@ -4117,16 +3835,16 @@
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="E7" s="18" t="n">
         <v>0.167</v>
@@ -4140,16 +3858,16 @@
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="E8" s="18" t="n">
         <v>0.167</v>
@@ -4163,16 +3881,16 @@
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="E9" s="18" t="n">
         <v>0.167</v>
@@ -4186,16 +3904,16 @@
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="E10" s="18" t="n">
         <v>0.167</v>
@@ -4209,16 +3927,16 @@
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="E11" s="18" t="n">
         <v>0.167</v>
@@ -4278,7 +3996,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -4309,60 +4027,60 @@
         <v>36</v>
       </c>
       <c r="D2" s="20" t="s">
+        <v>197</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>198</v>
+      </c>
+      <c r="F2" s="20" t="s">
+        <v>199</v>
+      </c>
+      <c r="G2" s="20" t="s">
+        <v>200</v>
+      </c>
+      <c r="H2" s="20" t="s">
+        <v>201</v>
+      </c>
+      <c r="I2" s="20" t="s">
+        <v>202</v>
+      </c>
+      <c r="J2" s="20" t="s">
+        <v>203</v>
+      </c>
+      <c r="K2" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="L2" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="M2" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="N2" s="20" t="s">
+        <v>207</v>
+      </c>
+      <c r="O2" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="P2" s="20" t="s">
         <v>209</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="Q2" s="20" t="s">
         <v>210</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="R2" s="20" t="s">
         <v>211</v>
-      </c>
-      <c r="G2" s="20" t="s">
-        <v>212</v>
-      </c>
-      <c r="H2" s="20" t="s">
-        <v>213</v>
-      </c>
-      <c r="I2" s="20" t="s">
-        <v>214</v>
-      </c>
-      <c r="J2" s="20" t="s">
-        <v>215</v>
-      </c>
-      <c r="K2" s="20" t="s">
-        <v>216</v>
-      </c>
-      <c r="L2" s="20" t="s">
-        <v>217</v>
-      </c>
-      <c r="M2" s="20" t="s">
-        <v>218</v>
-      </c>
-      <c r="N2" s="20" t="s">
-        <v>219</v>
-      </c>
-      <c r="O2" s="20" t="s">
-        <v>220</v>
-      </c>
-      <c r="P2" s="20" t="s">
-        <v>221</v>
-      </c>
-      <c r="Q2" s="20" t="s">
-        <v>222</v>
-      </c>
-      <c r="R2" s="20" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="D3" s="21" t="n">
         <v>8</v>
@@ -4375,28 +4093,28 @@
         <v>1</v>
       </c>
       <c r="G3" s="21" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="H3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="I3" s="21" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="J3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="K3" s="21" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="L3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="M3" s="21" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="N3" s="21" t="n">
         <v>6.5</v>
@@ -4471,7 +4189,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -4495,28 +4213,28 @@
         <v>36</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
       <c r="I2" s="20" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="J2" s="20" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="K2" s="20" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="XFB2" s="3"/>
       <c r="XFC2" s="3"/>
@@ -4524,29 +4242,29 @@
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="F3" s="21" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="G3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H3" s="21" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="I3" s="21" t="n">
         <v>0.5</v>
@@ -4560,29 +4278,29 @@
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="21" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>243</v>
+        <v>231</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="F4" s="21" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="G4" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H4" s="21" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="I4" s="21" t="n">
         <v>0.5</v>
@@ -4596,29 +4314,29 @@
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="21" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>245</v>
+        <v>233</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>246</v>
+        <v>234</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="F5" s="21" t="s">
-        <v>247</v>
+        <v>235</v>
       </c>
       <c r="G5" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="H5" s="21" t="s">
-        <v>248</v>
+        <v>236</v>
       </c>
       <c r="I5" s="21" t="n">
         <v>0.5</v>

</xml_diff>

<commit_message>
Add ROS bag loading in MATLAB
</commit_message>
<xml_diff>
--- a/src/flychams_common/config/Configuration-Multi-Agent.xlsx
+++ b/src/flychams_common/config/Configuration-Multi-Agent.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="Mission" sheetId="1" state="visible" r:id="rId3"/>
@@ -568,7 +568,7 @@
     <t xml:space="preserve">Tracking Window 1.1 Multi-Window (2 Windows)</t>
   </si>
   <si>
-    <t xml:space="preserve">(240x135)</t>
+    <t xml:space="preserve">(480x270)</t>
   </si>
   <si>
     <t xml:space="preserve">MULTIWINDOW01</t>
@@ -733,7 +733,7 @@
     <t xml:space="preserve">High-Resolution Central Camera</t>
   </si>
   <si>
-    <t xml:space="preserve">(1920x1080)</t>
+    <t xml:space="preserve">(3840x2160)</t>
   </si>
   <si>
     <t xml:space="preserve">(-0.08, 0.008, 0.0001, 0.002, -0.0015)</t>
@@ -781,7 +781,7 @@
     <numFmt numFmtId="165" formatCode="h:mm:ss"/>
     <numFmt numFmtId="166" formatCode="0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -849,6 +849,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -942,7 +948,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1019,6 +1025,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1028,6 +1038,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1852,92 +1866,92 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="C2" s="21" t="s">
         <v>237</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="F2" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="G2" s="20" t="s">
+      <c r="G2" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="H2" s="20" t="s">
+      <c r="H2" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="I2" s="20" t="s">
+      <c r="I2" s="21" t="s">
         <v>222</v>
       </c>
-      <c r="J2" s="20" t="s">
+      <c r="J2" s="21" t="s">
         <v>223</v>
       </c>
-      <c r="K2" s="20" t="s">
+      <c r="K2" s="21" t="s">
         <v>224</v>
       </c>
       <c r="L2" s="12"/>
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="22" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="22" t="s">
         <v>243</v>
       </c>
-      <c r="C3" s="21" t="b">
+      <c r="C3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="D3" s="22" t="s">
         <v>244</v>
       </c>
-      <c r="E3" s="21" t="b">
+      <c r="E3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="F3" s="21" t="s">
+      <c r="F3" s="22" t="s">
         <v>245</v>
       </c>
-      <c r="G3" s="21" t="b">
+      <c r="G3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="21" t="s">
+      <c r="H3" s="22" t="s">
         <v>246</v>
       </c>
-      <c r="I3" s="21" t="n">
+      <c r="I3" s="22" t="n">
         <v>0.4</v>
       </c>
-      <c r="J3" s="21" t="n">
+      <c r="J3" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="K3" s="21" t="n">
+      <c r="K3" s="22" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3751,7 +3765,7 @@
       <c r="C3" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="19" t="s">
         <v>179</v>
       </c>
       <c r="E3" s="18" t="n">
@@ -3774,7 +3788,7 @@
       <c r="C4" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="19" t="s">
         <v>179</v>
       </c>
       <c r="E4" s="18" t="n">
@@ -3797,7 +3811,7 @@
       <c r="C5" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="19" t="s">
         <v>179</v>
       </c>
       <c r="E5" s="18" t="n">
@@ -3820,7 +3834,7 @@
       <c r="C6" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="19" t="s">
         <v>179</v>
       </c>
       <c r="E6" s="18" t="n">
@@ -3843,7 +3857,7 @@
       <c r="C7" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="19" t="s">
         <v>179</v>
       </c>
       <c r="E7" s="18" t="n">
@@ -3866,7 +3880,7 @@
       <c r="C8" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="19" t="s">
         <v>179</v>
       </c>
       <c r="E8" s="18" t="n">
@@ -3889,7 +3903,7 @@
       <c r="C9" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="19" t="s">
         <v>179</v>
       </c>
       <c r="E9" s="18" t="n">
@@ -3912,7 +3926,7 @@
       <c r="C10" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" s="19" t="s">
         <v>179</v>
       </c>
       <c r="E10" s="18" t="n">
@@ -3935,7 +3949,7 @@
       <c r="C11" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="19" t="s">
         <v>179</v>
       </c>
       <c r="E11" s="18" t="n">
@@ -3995,140 +4009,140 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
-      <c r="O1" s="19"/>
-      <c r="P1" s="19"/>
-      <c r="Q1" s="19"/>
-      <c r="R1" s="19"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="C2" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="21" t="s">
         <v>197</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="21" t="s">
         <v>198</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="F2" s="21" t="s">
         <v>199</v>
       </c>
-      <c r="G2" s="20" t="s">
+      <c r="G2" s="21" t="s">
         <v>200</v>
       </c>
-      <c r="H2" s="20" t="s">
+      <c r="H2" s="21" t="s">
         <v>201</v>
       </c>
-      <c r="I2" s="20" t="s">
+      <c r="I2" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="J2" s="20" t="s">
+      <c r="J2" s="21" t="s">
         <v>203</v>
       </c>
-      <c r="K2" s="20" t="s">
+      <c r="K2" s="21" t="s">
         <v>204</v>
       </c>
-      <c r="L2" s="20" t="s">
+      <c r="L2" s="21" t="s">
         <v>205</v>
       </c>
-      <c r="M2" s="20" t="s">
+      <c r="M2" s="21" t="s">
         <v>206</v>
       </c>
-      <c r="N2" s="20" t="s">
+      <c r="N2" s="21" t="s">
         <v>207</v>
       </c>
-      <c r="O2" s="20" t="s">
+      <c r="O2" s="21" t="s">
         <v>208</v>
       </c>
-      <c r="P2" s="20" t="s">
+      <c r="P2" s="21" t="s">
         <v>209</v>
       </c>
-      <c r="Q2" s="20" t="s">
+      <c r="Q2" s="21" t="s">
         <v>210</v>
       </c>
-      <c r="R2" s="20" t="s">
+      <c r="R2" s="21" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="22" t="s">
         <v>212</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="22" t="s">
         <v>213</v>
       </c>
-      <c r="D3" s="21" t="n">
+      <c r="D3" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="E3" s="21" t="n">
+      <c r="E3" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="F3" s="21" t="b">
+      <c r="F3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="G3" s="21" t="s">
+      <c r="G3" s="22" t="s">
         <v>214</v>
       </c>
-      <c r="H3" s="21" t="b">
+      <c r="H3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="I3" s="21" t="s">
+      <c r="I3" s="22" t="s">
         <v>215</v>
       </c>
-      <c r="J3" s="21" t="b">
+      <c r="J3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="K3" s="21" t="s">
+      <c r="K3" s="22" t="s">
         <v>216</v>
       </c>
-      <c r="L3" s="21" t="b">
+      <c r="L3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="M3" s="21" t="s">
+      <c r="M3" s="22" t="s">
         <v>217</v>
       </c>
-      <c r="N3" s="21" t="n">
+      <c r="N3" s="22" t="n">
         <v>6.5</v>
       </c>
-      <c r="O3" s="21" t="n">
+      <c r="O3" s="22" t="n">
         <v>2.5</v>
       </c>
-      <c r="P3" s="21" t="n">
+      <c r="P3" s="22" t="n">
         <v>400</v>
       </c>
-      <c r="Q3" s="21" t="n">
+      <c r="Q3" s="22" t="n">
         <v>350</v>
       </c>
-      <c r="R3" s="21" t="n">
+      <c r="R3" s="22" t="n">
         <v>25</v>
       </c>
     </row>
@@ -4188,52 +4202,52 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="C2" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="21" t="s">
         <v>173</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="21" t="s">
         <v>218</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="F2" s="21" t="s">
         <v>219</v>
       </c>
-      <c r="G2" s="20" t="s">
+      <c r="G2" s="21" t="s">
         <v>220</v>
       </c>
-      <c r="H2" s="20" t="s">
+      <c r="H2" s="21" t="s">
         <v>221</v>
       </c>
-      <c r="I2" s="20" t="s">
+      <c r="I2" s="21" t="s">
         <v>222</v>
       </c>
-      <c r="J2" s="20" t="s">
+      <c r="J2" s="21" t="s">
         <v>223</v>
       </c>
-      <c r="K2" s="20" t="s">
+      <c r="K2" s="21" t="s">
         <v>224</v>
       </c>
       <c r="XFB2" s="3"/>
@@ -4241,110 +4255,110 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="22" t="s">
         <v>225</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="22" t="s">
         <v>226</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="D3" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="E3" s="21" t="s">
+      <c r="E3" s="22" t="s">
         <v>228</v>
       </c>
-      <c r="F3" s="21" t="s">
+      <c r="F3" s="22" t="s">
         <v>229</v>
       </c>
-      <c r="G3" s="21" t="b">
+      <c r="G3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="21" t="s">
+      <c r="H3" s="22" t="s">
         <v>230</v>
       </c>
-      <c r="I3" s="21" t="n">
+      <c r="I3" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="J3" s="21" t="n">
+      <c r="J3" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="K3" s="21" t="n">
+      <c r="K3" s="22" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="22" t="s">
         <v>231</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="22" t="s">
         <v>226</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="22" t="s">
         <v>232</v>
       </c>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="22" t="s">
         <v>228</v>
       </c>
-      <c r="F4" s="21" t="s">
+      <c r="F4" s="22" t="s">
         <v>229</v>
       </c>
-      <c r="G4" s="21" t="b">
+      <c r="G4" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H4" s="21" t="s">
+      <c r="H4" s="22" t="s">
         <v>230</v>
       </c>
-      <c r="I4" s="21" t="n">
+      <c r="I4" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="J4" s="21" t="n">
+      <c r="J4" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="21" t="n">
+      <c r="K4" s="22" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="22" t="s">
         <v>148</v>
       </c>
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="22" t="s">
         <v>233</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="22" t="s">
         <v>226</v>
       </c>
-      <c r="D5" s="21" t="s">
+      <c r="D5" s="23" t="s">
         <v>234</v>
       </c>
-      <c r="E5" s="21" t="s">
+      <c r="E5" s="22" t="s">
         <v>228</v>
       </c>
-      <c r="F5" s="21" t="s">
+      <c r="F5" s="22" t="s">
         <v>235</v>
       </c>
-      <c r="G5" s="21" t="b">
+      <c r="G5" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H5" s="21" t="s">
+      <c r="H5" s="22" t="s">
         <v>236</v>
       </c>
-      <c r="I5" s="21" t="n">
+      <c r="I5" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="J5" s="21" t="n">
+      <c r="J5" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="21" t="n">
+      <c r="K5" s="22" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add MATLAB doc and scripts
</commit_message>
<xml_diff>
--- a/src/flychams_common/config/Configuration-Multi-Agent.xlsx
+++ b/src/flychams_common/config/Configuration-Multi-Agent.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Mission" sheetId="1" state="visible" r:id="rId3"/>
@@ -64,6 +64,9 @@
     <t xml:space="preserve">StartHour</t>
   </si>
   <si>
+    <t xml:space="preserve">X</t>
+  </si>
+  <si>
     <t xml:space="preserve">MISSION00</t>
   </si>
   <si>
@@ -92,9 +95,6 @@
   </si>
   <si>
     <t xml:space="preserve">(16:30:00)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X</t>
   </si>
   <si>
     <t xml:space="preserve">MISSION01</t>
@@ -844,17 +844,18 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="2" tint="-0.75"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -948,7 +949,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -981,7 +982,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -993,12 +994,16 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1025,10 +1030,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1038,10 +1039,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1590,36 +1587,38 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8"/>
+      <c r="A3" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="B3" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L3" s="12"/>
       <c r="M3" s="12"/>
@@ -1668,9 +1667,7 @@
       <c r="BD3" s="12"/>
     </row>
     <row r="4" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
-        <v>21</v>
-      </c>
+      <c r="A4" s="13"/>
       <c r="B4" s="9" t="s">
         <v>22</v>
       </c>
@@ -1678,28 +1675,28 @@
         <v>23</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F4" s="11" t="s">
         <v>24</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L4" s="12"/>
       <c r="M4" s="12"/>
@@ -1756,28 +1753,28 @@
         <v>26</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" s="11" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L5" s="12"/>
       <c r="M5" s="12"/>
@@ -2005,12 +2002,12 @@
   </cols>
   <sheetData>
     <row r="1" s="7" customFormat="true" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
       <c r="E1" s="12"/>
       <c r="XFB1" s="3"/>
       <c r="XFC1" s="3"/>
@@ -2032,7 +2029,7 @@
     </row>
     <row r="3" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>30</v>
@@ -2040,7 +2037,7 @@
       <c r="C3" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="15" t="s">
         <v>32</v>
       </c>
     </row>
@@ -2054,7 +2051,7 @@
       <c r="C4" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="15" t="s">
         <v>35</v>
       </c>
     </row>
@@ -2094,15 +2091,15 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
@@ -2193,12 +2190,12 @@
         <v>41</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E3" s="15" t="n">
+      <c r="E3" s="16" t="n">
         <v>16</v>
       </c>
       <c r="F3" s="9" t="s">
@@ -2314,48 +2311,48 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="H2" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="I2" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="J2" s="18" t="s">
         <v>52</v>
       </c>
       <c r="L2" s="12"/>
@@ -2370,258 +2367,258 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" s="18" t="s">
+      <c r="C3" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="H3" s="18" t="n">
+      <c r="H3" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I3" s="18" t="n">
+      <c r="I3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="18" t="n">
+      <c r="J3" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="C4" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="18" t="s">
+      <c r="C4" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="F4" s="18" t="s">
+      <c r="F4" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="G4" s="18" t="s">
+      <c r="G4" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="H4" s="18" t="n">
+      <c r="H4" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I4" s="18" t="n">
+      <c r="I4" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="18" t="n">
+      <c r="J4" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="C5" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="18" t="s">
+      <c r="C5" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="H5" s="18" t="n">
+      <c r="H5" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I5" s="18" t="n">
+      <c r="I5" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J5" s="18" t="n">
+      <c r="J5" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="H6" s="18" t="n">
+      <c r="H6" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I6" s="18" t="n">
+      <c r="I6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="J6" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="G7" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="H7" s="18" t="n">
+      <c r="H7" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I7" s="18" t="n">
+      <c r="I7" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J7" s="18" t="n">
+      <c r="J7" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="F8" s="18" t="s">
+      <c r="F8" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="G8" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="H8" s="18" t="n">
+      <c r="H8" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I8" s="18" t="n">
+      <c r="I8" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="18" t="n">
+      <c r="J8" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="G9" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="H9" s="18" t="n">
+      <c r="H9" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I9" s="18" t="n">
+      <c r="I9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="18" t="n">
+      <c r="J9" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="G10" s="18" t="s">
+      <c r="G10" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="H10" s="18" t="n">
+      <c r="H10" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I10" s="18" t="n">
+      <c r="I10" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J10" s="18" t="n">
+      <c r="J10" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -2667,32 +2664,32 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="18" t="s">
         <v>85</v>
       </c>
       <c r="H2" s="12"/>
@@ -2708,22 +2705,22 @@
       <c r="XFD2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="D3" s="18" t="n">
+      <c r="D3" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E3" s="18" t="n">
+      <c r="E3" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F3" s="18" t="n">
+      <c r="F3" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G3" s="2"/>
@@ -2733,22 +2730,22 @@
       <c r="XEY3" s="3"/>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="D4" s="18" t="n">
+      <c r="D4" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="18" t="n">
+      <c r="E4" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F4" s="18" t="n">
+      <c r="F4" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G4" s="2"/>
@@ -2758,22 +2755,22 @@
       <c r="XEY4" s="3"/>
     </row>
     <row r="5" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="18" t="n">
+      <c r="D5" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G5" s="2"/>
@@ -2783,22 +2780,22 @@
       <c r="XEY5" s="3"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="D6" s="18" t="n">
+      <c r="D6" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F6" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G6" s="2"/>
@@ -2808,22 +2805,22 @@
       <c r="XEY6" s="3"/>
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="D7" s="18" t="n">
+      <c r="D7" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G7" s="2"/>
@@ -2833,22 +2830,22 @@
       <c r="XEY7" s="3"/>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="D8" s="18" t="n">
+      <c r="D8" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G8" s="2"/>
@@ -2858,22 +2855,22 @@
       <c r="XEY8" s="3"/>
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F9" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G9" s="2"/>
@@ -2883,22 +2880,22 @@
       <c r="XEY9" s="3"/>
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="D10" s="18" t="n">
+      <c r="D10" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E10" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F10" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G10" s="2"/>
@@ -2964,56 +2961,56 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="H2" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="I2" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="J2" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="K2" s="17" t="s">
+      <c r="K2" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="L2" s="17" t="s">
+      <c r="L2" s="18" t="s">
         <v>108</v>
       </c>
       <c r="M2" s="12"/>
@@ -3026,652 +3023,652 @@
       <c r="XFC2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="H3" s="18" t="s">
+      <c r="H3" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="I3" s="18" t="n">
+      <c r="I3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="18" t="n">
+      <c r="J3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K3" s="18" t="n">
+      <c r="K3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L3" s="18" t="s">
+      <c r="L3" s="19" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F4" s="18" t="s">
+      <c r="F4" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="G4" s="18" t="s">
+      <c r="G4" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="H4" s="18" t="s">
+      <c r="H4" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="I4" s="18" t="n">
+      <c r="I4" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J4" s="18" t="n">
+      <c r="J4" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K4" s="18" t="n">
+      <c r="K4" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L4" s="18" t="s">
+      <c r="L4" s="19" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="H5" s="18" t="s">
+      <c r="H5" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="I5" s="18" t="n">
+      <c r="I5" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J5" s="18" t="n">
+      <c r="J5" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K5" s="18" t="n">
+      <c r="K5" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L5" s="18" t="s">
+      <c r="L5" s="19" t="s">
         <v>127</v>
       </c>
       <c r="XFD5" s="12"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="H6" s="18" t="s">
+      <c r="H6" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="I6" s="18" t="n">
+      <c r="I6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="J6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K6" s="18" t="n">
+      <c r="K6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L6" s="18" t="s">
+      <c r="L6" s="19" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="G7" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="H7" s="18" t="s">
+      <c r="H7" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="I7" s="18" t="n">
+      <c r="I7" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J7" s="18" t="n">
+      <c r="J7" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K7" s="18" t="n">
+      <c r="K7" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L7" s="18" t="s">
+      <c r="L7" s="19" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F8" s="18" t="s">
+      <c r="F8" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="G8" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="H8" s="18" t="s">
+      <c r="H8" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="I8" s="18" t="n">
+      <c r="I8" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J8" s="18" t="n">
+      <c r="J8" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K8" s="18" t="n">
+      <c r="K8" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L8" s="18" t="s">
+      <c r="L8" s="19" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>137</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="19" t="s">
         <v>138</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="G9" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="H9" s="18" t="s">
+      <c r="H9" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="I9" s="18" t="n">
+      <c r="I9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="18" t="n">
+      <c r="J9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K9" s="18" t="n">
+      <c r="K9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L9" s="18" t="s">
+      <c r="L9" s="19" t="s">
         <v>139</v>
       </c>
       <c r="XFD9" s="2"/>
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="G10" s="18" t="s">
+      <c r="G10" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="H10" s="18" t="s">
+      <c r="H10" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="I10" s="18" t="n">
+      <c r="I10" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J10" s="18" t="n">
+      <c r="J10" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K10" s="18" t="n">
+      <c r="K10" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L10" s="18" t="s">
+      <c r="L10" s="19" t="s">
         <v>142</v>
       </c>
       <c r="XFD10" s="2"/>
     </row>
     <row r="11" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="E11" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="G11" s="18" t="s">
+      <c r="G11" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="H11" s="18" t="s">
+      <c r="H11" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="I11" s="18" t="n">
+      <c r="I11" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J11" s="18" t="n">
+      <c r="J11" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K11" s="18" t="n">
+      <c r="K11" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L11" s="18" t="s">
+      <c r="L11" s="19" t="s">
         <v>145</v>
       </c>
       <c r="XFD11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F12" s="18" t="s">
+      <c r="F12" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="G12" s="18" t="s">
+      <c r="G12" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="H12" s="18" t="s">
+      <c r="H12" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="I12" s="18" t="n">
+      <c r="I12" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J12" s="18" t="n">
+      <c r="J12" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K12" s="18" t="n">
+      <c r="K12" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L12" s="18" t="s">
+      <c r="L12" s="19" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="19" t="s">
         <v>150</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="19" t="s">
         <v>151</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="D13" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F13" s="18" t="s">
+      <c r="F13" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="G13" s="18" t="s">
+      <c r="G13" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="H13" s="18" t="s">
+      <c r="H13" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="I13" s="18" t="n">
+      <c r="I13" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J13" s="18" t="n">
+      <c r="J13" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K13" s="18" t="n">
+      <c r="K13" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L13" s="18" t="s">
+      <c r="L13" s="19" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="19" t="s">
         <v>153</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="D14" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="E14" s="18" t="s">
+      <c r="E14" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F14" s="18" t="s">
+      <c r="F14" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="G14" s="18" t="s">
+      <c r="G14" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="H14" s="18" t="s">
+      <c r="H14" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="I14" s="18" t="n">
+      <c r="I14" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J14" s="18" t="n">
+      <c r="J14" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K14" s="18" t="n">
+      <c r="K14" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L14" s="18" t="s">
+      <c r="L14" s="19" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="19" t="s">
         <v>156</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="19" t="s">
         <v>157</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="D15" s="18" t="s">
+      <c r="D15" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="E15" s="18" t="s">
+      <c r="E15" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F15" s="18" t="s">
+      <c r="F15" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="G15" s="18" t="s">
+      <c r="G15" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="H15" s="18" t="s">
+      <c r="H15" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="I15" s="18" t="n">
+      <c r="I15" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J15" s="18" t="n">
+      <c r="J15" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K15" s="18" t="n">
+      <c r="K15" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L15" s="18" t="s">
+      <c r="L15" s="19" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="s">
+      <c r="A16" s="19" t="s">
         <v>159</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="E16" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F16" s="18" t="s">
+      <c r="F16" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="G16" s="18" t="s">
+      <c r="G16" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="H16" s="18" t="s">
+      <c r="H16" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="I16" s="18" t="n">
+      <c r="I16" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J16" s="18" t="n">
+      <c r="J16" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K16" s="18" t="n">
+      <c r="K16" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L16" s="18" t="s">
+      <c r="L16" s="19" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="19" t="s">
         <v>162</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="19" t="s">
         <v>163</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="D17" s="18" t="s">
+      <c r="D17" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="E17" s="18" t="s">
+      <c r="E17" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F17" s="18" t="s">
+      <c r="F17" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="G17" s="18" t="s">
+      <c r="G17" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="H17" s="18" t="s">
+      <c r="H17" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="I17" s="18" t="n">
+      <c r="I17" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J17" s="18" t="n">
+      <c r="J17" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K17" s="18" t="n">
+      <c r="K17" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L17" s="18" t="s">
+      <c r="L17" s="19" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="19" t="s">
         <v>165</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="B18" s="19" t="s">
         <v>166</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="D18" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="E18" s="18" t="s">
+      <c r="E18" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F18" s="18" t="s">
+      <c r="F18" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="G18" s="18" t="s">
+      <c r="G18" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="H18" s="18" t="s">
+      <c r="H18" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="I18" s="18" t="n">
+      <c r="I18" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J18" s="18" t="n">
+      <c r="J18" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K18" s="18" t="n">
+      <c r="K18" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L18" s="18" t="s">
+      <c r="L18" s="19" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="19" t="s">
         <v>170</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="19" t="s">
         <v>171</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="C19" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="D19" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="E19" s="18" t="s">
+      <c r="E19" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="F19" s="18" t="s">
+      <c r="F19" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="G19" s="18" t="s">
+      <c r="G19" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="H19" s="18" t="s">
+      <c r="H19" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="I19" s="18" t="n">
+      <c r="I19" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J19" s="18" t="n">
+      <c r="J19" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K19" s="18" t="n">
+      <c r="K19" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L19" s="18" t="s">
+      <c r="L19" s="19" t="s">
         <v>172</v>
       </c>
     </row>
@@ -3712,36 +3709,36 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="18" t="s">
         <v>174</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="18" t="s">
         <v>176</v>
       </c>
       <c r="XEU2" s="3"/>
@@ -3756,209 +3753,209 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>177</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>178</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="19" t="s">
         <v>93</v>
       </c>
       <c r="D3" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="E3" s="18" t="n">
+      <c r="E3" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F3" s="18" t="n">
+      <c r="F3" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="18" t="n">
+      <c r="G3" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>180</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>93</v>
       </c>
       <c r="D4" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="E4" s="18" t="n">
+      <c r="E4" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F4" s="18" t="n">
+      <c r="F4" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="18" t="n">
+      <c r="G4" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>182</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="19" t="s">
         <v>95</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="18" t="n">
+      <c r="G5" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>184</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>185</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="19" t="s">
         <v>95</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F6" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="18" t="n">
+      <c r="G6" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="19" t="s">
         <v>186</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>187</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>97</v>
       </c>
       <c r="D7" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="18" t="n">
+      <c r="G7" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="19" t="s">
         <v>188</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="19" t="s">
         <v>97</v>
       </c>
       <c r="D8" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="18" t="n">
+      <c r="G8" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>190</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="19" t="s">
         <v>191</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="19" t="s">
         <v>101</v>
       </c>
       <c r="D9" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F9" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="18" t="n">
+      <c r="G9" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="19" t="s">
         <v>192</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="19" t="s">
         <v>101</v>
       </c>
       <c r="D10" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E10" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F10" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="18" t="n">
+      <c r="G10" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="19" t="s">
         <v>194</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="19" t="s">
         <v>195</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="19" t="s">
         <v>101</v>
       </c>
       <c r="D11" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="E11" s="18" t="n">
+      <c r="E11" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F11" s="18" t="n">
+      <c r="F11" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="18" t="n">
+      <c r="G11" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
@@ -4336,7 +4333,7 @@
       <c r="C5" s="22" t="s">
         <v>226</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="22" t="s">
         <v>234</v>
       </c>
       <c r="E5" s="22" t="s">

</xml_diff>

<commit_message>
Add assignment benchmark configuration
</commit_message>
<xml_diff>
--- a/src/flychams_common/config/Configuration-Multi-Agent.xlsx
+++ b/src/flychams_common/config/Configuration-Multi-Agent.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Mission" sheetId="1" state="visible" r:id="rId3"/>
@@ -373,7 +373,7 @@
     <t xml:space="preserve">Central</t>
   </si>
   <si>
-    <t xml:space="preserve">(X=0.0, Y=0.0, Z=-0.05)</t>
+    <t xml:space="preserve">(X=0.0, Y=0.0, Z=-0.08)</t>
   </si>
   <si>
     <t xml:space="preserve">(Roll=0.0, Pitch=90.0, Yaw=90.0)</t>
@@ -394,7 +394,7 @@
     <t xml:space="preserve">Tracking</t>
   </si>
   <si>
-    <t xml:space="preserve">(X=0.3, Y=0.0, Z=-0.05)</t>
+    <t xml:space="preserve">(X=0.19, Y=0.0, Z=-0.04)</t>
   </si>
   <si>
     <t xml:space="preserve">(Roll=0.0, Pitch=90.0, Yaw=0.0)</t>
@@ -409,7 +409,7 @@
     <t xml:space="preserve">Tracking Head 1.2 Multi-Camera (2 Cameras)</t>
   </si>
   <si>
-    <t xml:space="preserve">(X=0.0, Y=0.3, Z=-0.05)</t>
+    <t xml:space="preserve">(X=-0.19, Y=0.0, Z=-0.04)</t>
   </si>
   <si>
     <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT00/MULTICAMERA02</t>
@@ -532,7 +532,35 @@
     <t xml:space="preserve">Tracking Head 1.3 Multi-Camera (3 Cameras)</t>
   </si>
   <si>
-    <t xml:space="preserve">(X=-0.3, Y=0.0, Z=-0.05)</t>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(X=0.0, Y=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">0.19</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, Z=-0.04)</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">(Roll=0.0, Pitch=90.0, Yaw=180.0)</t>
@@ -776,10 +804,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="h:mm:ss"/>
     <numFmt numFmtId="166" formatCode="0"/>
+    <numFmt numFmtId="167" formatCode="General"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -844,18 +873,17 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="16"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color theme="2" tint="-0.75"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -982,7 +1010,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -994,16 +1022,12 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1039,6 +1063,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1352,37 +1380,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="44546a"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="e7e6e6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4472c4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="ed7d31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="a5a5a5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="ffc000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="5b9bd5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="70ad47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0563c1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="954f72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office 2013 - 2022">
@@ -1522,7 +1550,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:XFD9"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="21" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="21" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.44"/>
@@ -1667,7 +1695,7 @@
       <c r="BD3" s="12"/>
     </row>
     <row r="4" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13"/>
+      <c r="A4" s="8"/>
       <c r="B4" s="9" t="s">
         <v>22</v>
       </c>
@@ -1849,7 +1877,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="2" width="29.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="40.25"/>
@@ -1863,92 +1891,92 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>196</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>237</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>238</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>240</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>241</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="20" t="s">
         <v>242</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="20" t="s">
         <v>223</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="20" t="s">
         <v>224</v>
       </c>
       <c r="L2" s="12"/>
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>243</v>
       </c>
       <c r="C3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="21" t="s">
         <v>244</v>
       </c>
       <c r="E3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="21" t="s">
         <v>245</v>
       </c>
       <c r="G3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="21" t="s">
         <v>246</v>
       </c>
-      <c r="I3" s="22" t="n">
+      <c r="I3" s="21" t="n">
         <v>0.4</v>
       </c>
-      <c r="J3" s="22" t="n">
+      <c r="J3" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="K3" s="22" t="n">
+      <c r="K3" s="21" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1989,7 +2017,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="33.54"/>
@@ -2002,12 +2030,12 @@
   </cols>
   <sheetData>
     <row r="1" s="7" customFormat="true" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
       <c r="E1" s="12"/>
       <c r="XFB1" s="3"/>
       <c r="XFC1" s="3"/>
@@ -2037,7 +2065,7 @@
       <c r="C3" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="14" t="s">
         <v>32</v>
       </c>
     </row>
@@ -2051,7 +2079,7 @@
       <c r="C4" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="14" t="s">
         <v>35</v>
       </c>
     </row>
@@ -2080,7 +2108,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:BM1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="38.38"/>
@@ -2091,15 +2119,15 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
@@ -2195,7 +2223,7 @@
       <c r="D3" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E3" s="16" t="n">
+      <c r="E3" s="15" t="n">
         <v>16</v>
       </c>
       <c r="F3" s="9" t="s">
@@ -2292,7 +2320,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD13"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="38.28"/>
@@ -2311,48 +2339,48 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="17" t="s">
         <v>52</v>
       </c>
       <c r="L2" s="12"/>
@@ -2367,258 +2395,258 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="H3" s="19" t="n">
+      <c r="H3" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I3" s="19" t="n">
+      <c r="I3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="19" t="n">
+      <c r="J3" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="H4" s="19" t="n">
+      <c r="H4" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I4" s="19" t="n">
+      <c r="I4" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="19" t="n">
+      <c r="J4" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="H5" s="19" t="n">
+      <c r="H5" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I5" s="19" t="n">
+      <c r="I5" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J5" s="19" t="n">
+      <c r="J5" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="H6" s="19" t="n">
+      <c r="H6" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I6" s="19" t="n">
+      <c r="I6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="19" t="n">
+      <c r="J6" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="H7" s="19" t="n">
+      <c r="H7" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I7" s="19" t="n">
+      <c r="I7" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J7" s="19" t="n">
+      <c r="J7" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="H8" s="19" t="n">
+      <c r="H8" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="I8" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="19" t="n">
+      <c r="J8" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="H9" s="19" t="n">
+      <c r="H9" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="I9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="J9" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="G10" s="19" t="s">
+      <c r="G10" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="H10" s="19" t="n">
+      <c r="H10" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="I10" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J10" s="19" t="n">
+      <c r="J10" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -2648,7 +2676,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="38.28"/>
@@ -2664,32 +2692,32 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>85</v>
       </c>
       <c r="H2" s="12"/>
@@ -2705,22 +2733,22 @@
       <c r="XFD2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="D3" s="19" t="n">
+      <c r="D3" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E3" s="19" t="n">
+      <c r="E3" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F3" s="19" t="n">
+      <c r="F3" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G3" s="2"/>
@@ -2730,22 +2758,22 @@
       <c r="XEY3" s="3"/>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="D4" s="19" t="n">
+      <c r="D4" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="19" t="n">
+      <c r="E4" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F4" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G4" s="2"/>
@@ -2755,22 +2783,22 @@
       <c r="XEY4" s="3"/>
     </row>
     <row r="5" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F5" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G5" s="2"/>
@@ -2780,22 +2808,22 @@
       <c r="XEY5" s="3"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F6" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G6" s="2"/>
@@ -2805,22 +2833,22 @@
       <c r="XEY6" s="3"/>
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F7" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G7" s="2"/>
@@ -2830,22 +2858,22 @@
       <c r="XEY7" s="3"/>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E8" s="19" t="n">
+      <c r="E8" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F8" s="19" t="n">
+      <c r="F8" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G8" s="2"/>
@@ -2855,22 +2883,22 @@
       <c r="XEY8" s="3"/>
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G9" s="2"/>
@@ -2880,22 +2908,22 @@
       <c r="XEY9" s="3"/>
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E10" s="19" t="n">
+      <c r="E10" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F10" s="19" t="n">
+      <c r="F10" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G10" s="2"/>
@@ -2943,7 +2971,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD19"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="45.28"/>
@@ -2961,56 +2989,56 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="K2" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="L2" s="18" t="s">
+      <c r="L2" s="17" t="s">
         <v>108</v>
       </c>
       <c r="M2" s="12"/>
@@ -3023,652 +3051,652 @@
       <c r="XFC2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="I3" s="19" t="n">
+      <c r="I3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="19" t="n">
+      <c r="J3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K3" s="19" t="n">
+      <c r="K3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L3" s="19" t="s">
+      <c r="L3" s="18" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>118</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="H4" s="19" t="s">
+      <c r="H4" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="I4" s="19" t="n">
+      <c r="I4" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J4" s="19" t="n">
+      <c r="J4" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K4" s="19" t="n">
+      <c r="K4" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L4" s="19" t="s">
+      <c r="L4" s="18" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="I5" s="19" t="n">
+      <c r="I5" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J5" s="19" t="n">
+      <c r="J5" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K5" s="19" t="n">
+      <c r="K5" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L5" s="19" t="s">
+      <c r="L5" s="18" t="s">
         <v>127</v>
       </c>
       <c r="XFD5" s="12"/>
     </row>
     <row r="6" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>128</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="H6" s="19" t="s">
+      <c r="H6" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="I6" s="19" t="n">
+      <c r="I6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="19" t="n">
+      <c r="J6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K6" s="19" t="n">
+      <c r="K6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L6" s="19" t="s">
+      <c r="L6" s="18" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="7" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="H7" s="19" t="s">
+      <c r="H7" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="I7" s="19" t="n">
+      <c r="I7" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J7" s="19" t="n">
+      <c r="J7" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K7" s="19" t="n">
+      <c r="K7" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L7" s="19" t="s">
+      <c r="L7" s="18" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="8" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="H8" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="I8" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J8" s="19" t="n">
+      <c r="J8" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K8" s="19" t="n">
+      <c r="K8" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L8" s="19" t="s">
+      <c r="L8" s="18" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="9" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>137</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="H9" s="19" t="s">
+      <c r="H9" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="I9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="J9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K9" s="19" t="n">
+      <c r="K9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L9" s="19" t="s">
+      <c r="L9" s="18" t="s">
         <v>139</v>
       </c>
       <c r="XFD9" s="2"/>
     </row>
     <row r="10" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="G10" s="19" t="s">
+      <c r="G10" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="H10" s="19" t="s">
+      <c r="H10" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="I10" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J10" s="19" t="n">
+      <c r="J10" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K10" s="19" t="n">
+      <c r="K10" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L10" s="19" t="s">
+      <c r="L10" s="18" t="s">
         <v>142</v>
       </c>
       <c r="XFD10" s="2"/>
     </row>
     <row r="11" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="18" t="s">
         <v>144</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="H11" s="19" t="s">
+      <c r="H11" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="I11" s="19" t="n">
+      <c r="I11" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="J11" s="19" t="n">
+      <c r="J11" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K11" s="19" t="n">
+      <c r="K11" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L11" s="19" t="s">
+      <c r="L11" s="18" t="s">
         <v>145</v>
       </c>
       <c r="XFD11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E12" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="F12" s="19" t="s">
+      <c r="F12" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="G12" s="19" t="s">
+      <c r="G12" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="H12" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="I12" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="J12" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="K12" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="L12" s="18" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="F13" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="G13" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="H13" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="I13" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="J13" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="L13" s="18" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="F14" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="G14" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="H14" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="I14" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="J14" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="K14" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="L14" s="18" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="F15" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="G15" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="H12" s="19" t="s">
+      <c r="H15" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="I12" s="19" t="n">
+      <c r="I15" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J12" s="19" t="n">
+      <c r="J15" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K12" s="19" t="n">
+      <c r="K15" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L12" s="19" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
-        <v>150</v>
-      </c>
-      <c r="B13" s="19" t="s">
-        <v>151</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>95</v>
-      </c>
-      <c r="D13" s="19" t="s">
+      <c r="L15" s="18" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18" t="s">
+        <v>159</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="E16" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="F16" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="G16" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="H16" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="I16" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="K16" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="L16" s="18" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="s">
+        <v>162</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="F17" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="G17" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="H17" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="I17" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="K17" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="L17" s="18" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="18" t="s">
+        <v>165</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="F18" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="G18" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="H18" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="I18" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="K18" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="L18" s="18" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="D19" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E19" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F19" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="G13" s="19" t="s">
-        <v>114</v>
-      </c>
-      <c r="H13" s="19" t="s">
+      <c r="G19" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="H19" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="I13" s="19" t="n">
+      <c r="I19" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J13" s="19" t="n">
+      <c r="J19" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K13" s="19" t="n">
+      <c r="K19" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L13" s="19" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
-        <v>153</v>
-      </c>
-      <c r="B14" s="19" t="s">
-        <v>154</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>97</v>
-      </c>
-      <c r="D14" s="19" t="s">
-        <v>148</v>
-      </c>
-      <c r="E14" s="19" t="s">
-        <v>112</v>
-      </c>
-      <c r="F14" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="G14" s="19" t="s">
-        <v>114</v>
-      </c>
-      <c r="H14" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="I14" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="J14" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="K14" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="L14" s="19" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
-        <v>156</v>
-      </c>
-      <c r="B15" s="19" t="s">
-        <v>157</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="D15" s="19" t="s">
-        <v>111</v>
-      </c>
-      <c r="E15" s="19" t="s">
-        <v>112</v>
-      </c>
-      <c r="F15" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="G15" s="19" t="s">
-        <v>114</v>
-      </c>
-      <c r="H15" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="I15" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="J15" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="K15" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="L15" s="19" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="B16" s="19" t="s">
-        <v>160</v>
-      </c>
-      <c r="C16" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="D16" s="19" t="s">
-        <v>119</v>
-      </c>
-      <c r="E16" s="19" t="s">
-        <v>112</v>
-      </c>
-      <c r="F16" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="G16" s="19" t="s">
-        <v>121</v>
-      </c>
-      <c r="H16" s="19" t="s">
-        <v>122</v>
-      </c>
-      <c r="I16" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="K16" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="L16" s="19" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
-        <v>162</v>
-      </c>
-      <c r="B17" s="19" t="s">
-        <v>163</v>
-      </c>
-      <c r="C17" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="D17" s="19" t="s">
-        <v>119</v>
-      </c>
-      <c r="E17" s="19" t="s">
-        <v>112</v>
-      </c>
-      <c r="F17" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="G17" s="19" t="s">
-        <v>126</v>
-      </c>
-      <c r="H17" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="I17" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="K17" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="L17" s="19" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="B18" s="19" t="s">
-        <v>166</v>
-      </c>
-      <c r="C18" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>119</v>
-      </c>
-      <c r="E18" s="19" t="s">
-        <v>112</v>
-      </c>
-      <c r="F18" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="G18" s="19" t="s">
-        <v>167</v>
-      </c>
-      <c r="H18" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="I18" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="K18" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="L18" s="19" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
-        <v>170</v>
-      </c>
-      <c r="B19" s="19" t="s">
-        <v>171</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>148</v>
-      </c>
-      <c r="E19" s="19" t="s">
-        <v>112</v>
-      </c>
-      <c r="F19" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="G19" s="19" t="s">
-        <v>114</v>
-      </c>
-      <c r="H19" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="I19" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="J19" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="K19" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="L19" s="19" t="s">
+      <c r="L19" s="18" t="s">
         <v>172</v>
       </c>
     </row>
@@ -3695,7 +3723,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD17"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="57.21"/>
@@ -3709,36 +3737,36 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>174</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>176</v>
       </c>
       <c r="XEU2" s="3"/>
@@ -3753,209 +3781,209 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="E3" s="19" t="n">
+      <c r="E3" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F3" s="19" t="n">
+      <c r="F3" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="19" t="n">
+      <c r="G3" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>180</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="E4" s="19" t="n">
+      <c r="E4" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F4" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="19" t="n">
+      <c r="G4" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>182</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F5" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="19" t="n">
+      <c r="G5" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>185</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F6" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="19" t="n">
+      <c r="G6" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F7" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="19" t="n">
+      <c r="G7" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>188</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>189</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="E8" s="19" t="n">
+      <c r="E8" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F8" s="19" t="n">
+      <c r="F8" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="19" t="n">
+      <c r="G8" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="18" t="s">
         <v>190</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="19" t="n">
+      <c r="G9" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="18" t="s">
         <v>192</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="E10" s="19" t="n">
+      <c r="E10" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F10" s="19" t="n">
+      <c r="F10" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="19" t="n">
+      <c r="G10" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="E11" s="19" t="n">
+      <c r="E11" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F11" s="19" t="n">
+      <c r="F11" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="19" t="n">
+      <c r="G11" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
@@ -3988,7 +4016,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:R1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="34.63"/>
@@ -4006,140 +4034,140 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>196</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="20"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
+      <c r="P1" s="19"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="19"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>197</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>200</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="20" t="s">
         <v>201</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="20" t="s">
         <v>202</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="20" t="s">
         <v>203</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="20" t="s">
         <v>204</v>
       </c>
-      <c r="L2" s="21" t="s">
+      <c r="L2" s="20" t="s">
         <v>205</v>
       </c>
-      <c r="M2" s="21" t="s">
+      <c r="M2" s="20" t="s">
         <v>206</v>
       </c>
-      <c r="N2" s="21" t="s">
+      <c r="N2" s="20" t="s">
         <v>207</v>
       </c>
-      <c r="O2" s="21" t="s">
+      <c r="O2" s="20" t="s">
         <v>208</v>
       </c>
-      <c r="P2" s="21" t="s">
+      <c r="P2" s="20" t="s">
         <v>209</v>
       </c>
-      <c r="Q2" s="21" t="s">
+      <c r="Q2" s="20" t="s">
         <v>210</v>
       </c>
-      <c r="R2" s="21" t="s">
+      <c r="R2" s="20" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>212</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="21" t="s">
         <v>213</v>
       </c>
-      <c r="D3" s="22" t="n">
+      <c r="D3" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="E3" s="22" t="n">
+      <c r="E3" s="21" t="n">
         <v>12</v>
       </c>
       <c r="F3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="G3" s="21" t="s">
         <v>214</v>
       </c>
       <c r="H3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="I3" s="22" t="s">
+      <c r="I3" s="21" t="s">
         <v>215</v>
       </c>
       <c r="J3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="K3" s="22" t="s">
+      <c r="K3" s="21" t="s">
         <v>216</v>
       </c>
       <c r="L3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="M3" s="22" t="s">
+      <c r="M3" s="21" t="s">
         <v>217</v>
       </c>
-      <c r="N3" s="22" t="n">
+      <c r="N3" s="21" t="n">
         <v>6.5</v>
       </c>
-      <c r="O3" s="22" t="n">
+      <c r="O3" s="21" t="n">
         <v>2.5</v>
       </c>
-      <c r="P3" s="22" t="n">
+      <c r="P3" s="21" t="n">
         <v>400</v>
       </c>
-      <c r="Q3" s="22" t="n">
+      <c r="Q3" s="21" t="n">
         <v>350</v>
       </c>
-      <c r="R3" s="22" t="n">
+      <c r="R3" s="21" t="n">
         <v>25</v>
       </c>
     </row>
@@ -4183,7 +4211,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:XFD1048576"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="26.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="63.93"/>
@@ -4199,52 +4227,52 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>196</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>173</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>218</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>219</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>220</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="20" t="s">
         <v>221</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="20" t="s">
         <v>223</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="20" t="s">
         <v>224</v>
       </c>
       <c r="XFB2" s="3"/>
@@ -4252,110 +4280,110 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>225</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="21" t="s">
         <v>226</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="21" t="s">
         <v>227</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="E3" s="21" t="s">
         <v>228</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="21" t="s">
         <v>229</v>
       </c>
       <c r="G3" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="21" t="s">
         <v>230</v>
       </c>
-      <c r="I3" s="22" t="n">
+      <c r="I3" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="J3" s="22" t="n">
+      <c r="J3" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K3" s="22" t="n">
+      <c r="K3" s="21" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>119</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="21" t="s">
         <v>231</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="21" t="s">
         <v>226</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="21" t="s">
         <v>232</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="21" t="s">
         <v>228</v>
       </c>
-      <c r="F4" s="22" t="s">
+      <c r="F4" s="21" t="s">
         <v>229</v>
       </c>
       <c r="G4" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H4" s="22" t="s">
+      <c r="H4" s="21" t="s">
         <v>230</v>
       </c>
-      <c r="I4" s="22" t="n">
+      <c r="I4" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="J4" s="22" t="n">
+      <c r="J4" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="22" t="n">
+      <c r="K4" s="21" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="21" t="s">
         <v>233</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="21" t="s">
         <v>226</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="21" t="s">
         <v>234</v>
       </c>
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="21" t="s">
         <v>228</v>
       </c>
-      <c r="F5" s="22" t="s">
+      <c r="F5" s="21" t="s">
         <v>235</v>
       </c>
       <c r="G5" s="22" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H5" s="22" t="s">
+      <c r="H5" s="21" t="s">
         <v>236</v>
       </c>
-      <c r="I5" s="22" t="n">
+      <c r="I5" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="J5" s="22" t="n">
+      <c r="J5" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="22" t="n">
+      <c r="K5" s="21" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>